<commit_message>
added check on binaries
</commit_message>
<xml_diff>
--- a/plants_data/technologies.xlsx
+++ b/plants_data/technologies.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\plants_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8ADF3C3-D111-433F-8B81-6B6AD1E5BB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04977281-1E61-438D-A525-1E964F7F9B9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4020" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
SMR, feedgas mixer, eSMR
</commit_message>
<xml_diff>
--- a/plants_data/technologies.xlsx
+++ b/plants_data/technologies.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\plants_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B80DBD-2C89-47F1-B8E8-FF3B3FDA14D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26B9374-725F-4248-A972-565DCAACFFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-360" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="existing" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="25">
   <si>
     <t>cluster</t>
   </si>
@@ -98,6 +98,9 @@
   </si>
   <si>
     <t>WGS_syngas</t>
+  </si>
+  <si>
+    <t>feedgas_mixer</t>
   </si>
 </sst>
 </file>
@@ -415,10 +418,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -473,8 +476,11 @@
       <c r="R1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -529,8 +535,11 @@
       <c r="R2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -585,8 +594,11 @@
       <c r="R3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -641,8 +653,11 @@
       <c r="R4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -697,8 +712,11 @@
       <c r="R5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -753,8 +771,11 @@
       <c r="R6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -807,6 +828,9 @@
         <v>0</v>
       </c>
       <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
         <v>0</v>
       </c>
     </row>
@@ -817,10 +841,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD6448D7-10EE-4973-BCA6-F7E0B963E195}">
-  <dimension ref="A1:R7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -875,8 +899,11 @@
       <c r="R1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -931,8 +958,11 @@
       <c r="R2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -987,8 +1017,11 @@
       <c r="R3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1043,8 +1076,11 @@
       <c r="R4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -1099,8 +1135,11 @@
       <c r="R5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -1155,8 +1194,11 @@
       <c r="R6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="S6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -1209,6 +1251,9 @@
         <v>1</v>
       </c>
       <c r="R7">
+        <v>1</v>
+      </c>
+      <c r="S7">
         <v>1</v>
       </c>
     </row>

</xml_diff>